<commit_message>
Add Canada, Australia and UAE: 14 universities, country rules, QS 2027 ranks in finder and Excel; extend FAQ; add other destinations (Singapore, Russia, China, Japan) to Statistics
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RHDSLk4ybyUqj4e2g7Ubep
</commit_message>
<xml_diff>
--- a/site/downloads/BiswaPath_University_Guide_2027.xlsx
+++ b/site/downloads/BiswaPath_University_Guide_2027.xlsx
@@ -22,9 +22,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="297">
-  <si>
-    <t xml:space="preserve">BiswaPath – University Guide (first 35 universities)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="421">
+  <si>
+    <t xml:space="preserve">BiswaPath – University Guide (49 universities)</t>
   </si>
   <si>
     <t xml:space="preserve">Compiled 19 October 2026. Every fee and date links to the page it came from. Always confirm on the university's own website before applying.</t>
@@ -36,7 +36,7 @@
     <t xml:space="preserve">• 'Universities' – one row per university: application fee, deadlines, example tuition, scholarships, a link to chat with current students, and Indian/Bengali/Bangladeshi student societies.</t>
   </si>
   <si>
-    <t xml:space="preserve">• 'Country rules' – rules that apply to every university in a country (UCAS, uni-assist, Swedish national admissions, US applications) and how PhDs work there.</t>
+    <t xml:space="preserve">• 'Country rules' – rules that apply to every university in a country (UCAS, uni-assist, Swedish national admissions, US, Canadian, Australian and UAE applications) and how PhDs work there.</t>
   </si>
   <si>
     <t xml:space="preserve">• Blank cells mean we have not yet verified that information – not that it does not exist.</t>
@@ -90,6 +90,9 @@
     <t xml:space="preserve">PhD – how it works</t>
   </si>
   <si>
+    <t xml:space="preserve">QS World University Rankings 2027</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chat with current students</t>
   </si>
   <si>
@@ -126,6 +129,9 @@
     <t xml:space="preserve">Funded PhDs (studentships) are advertised on each university's research pages and on FindAPhD; most UK funding deadlines fall between December and March.</t>
   </si>
   <si>
+    <t xml:space="preserve">Not in QS top 100</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.coventry.ac.uk/unibuddy/</t>
   </si>
   <si>
@@ -150,6 +156,9 @@
     <t xml:space="preserve">Inspiring Excellence £5,000 or £10,000 (overseas, self-funded); rounds 7 Dec 2026, 15 Mar 2027, 1 May 2027</t>
   </si>
   <si>
+    <t xml:space="preserve">85</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://dur.ac.uk/study/student-connect/unibuddy/</t>
   </si>
   <si>
@@ -195,6 +204,9 @@
     <t xml:space="preserve">e.g. Physics MSc £38,100 (international, 2027/28)</t>
   </si>
   <si>
+    <t xml:space="preserve">37</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.kcl.ac.uk/study/postgraduate-taught/offer-holders/subjects</t>
   </si>
   <si>
@@ -213,6 +225,9 @@
     <t xml:space="preserve">£95 online application fee (per LSE e-shop)</t>
   </si>
   <si>
+    <t xml:space="preserve">62</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.lse.ac.uk/study-at-lse/chat-to-our-students</t>
   </si>
   <si>
@@ -318,6 +333,9 @@
     <t xml:space="preserve">£60 only for Business School and Economics taught Master's (2027/28); waiver for nationals of medium/low HDI countries (India and Bangladesh are medium HDI – check)</t>
   </si>
   <si>
+    <t xml:space="preserve">57</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.bristol.ac.uk/study/postgraduate/visits-open-days/postgraduate-chats/</t>
   </si>
   <si>
@@ -348,6 +366,9 @@
     <t xml:space="preserve">Gates Cambridge (funding deadline 8 Dec 2026 for most applicants)</t>
   </si>
   <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.postgraduate.study.cam.ac.uk/international/chat-our-students</t>
   </si>
   <si>
@@ -369,6 +390,9 @@
     <t xml:space="preserve">See programme page</t>
   </si>
   <si>
+    <t xml:space="preserve">35</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://study.ed.ac.uk/chat-to-our-students</t>
   </si>
   <si>
@@ -387,6 +411,9 @@
     <t xml:space="preserve">Six application rounds per cycle; places may become limited from 16 December</t>
   </si>
   <si>
+    <t xml:space="preserve">80</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.gla.ac.uk/study/studentlife/askastudent/askastudentenquiryform</t>
   </si>
   <si>
@@ -480,6 +507,9 @@
     <t xml:space="preserve">Set per course; main funding deadlines Dec/Jan – see course page</t>
   </si>
   <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://ox.ac.uk/node/7038428</t>
   </si>
   <si>
@@ -576,6 +606,9 @@
     <t xml:space="preserve">PhDs are often paid research posts; search the DAAD PhD database and university job pages.</t>
   </si>
   <si>
+    <t xml:space="preserve">86</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://migaku.com/blog/language-fun/tum-lmu-heidelberg-tuition-guide-for-international-students</t>
   </si>
   <si>
@@ -594,6 +627,9 @@
     <t xml:space="preserve">No general tuition for international students (some programmes charge, e.g. PPE €5,250/semester)</t>
   </si>
   <si>
+    <t xml:space="preserve">61</t>
+  </si>
+  <si>
     <t xml:space="preserve">Munich Indian Students Association (MISA): https://www.misa.hsg.fs.tum.de/</t>
   </si>
   <si>
@@ -654,6 +690,9 @@
     <t xml:space="preserve">Non-EU: Master's usually €4,000 or €6,000 per semester (rising to €4,600/€6,800 from WS 2027/28)</t>
   </si>
   <si>
+    <t xml:space="preserve">25</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.mygermanuniversity.com/universities/Technical-University-of-Munich/application-deadlines ; https://www.gradgermany.com/blog/germany-tuition-fees-by-state-2026</t>
   </si>
   <si>
@@ -711,6 +750,9 @@
     <t xml:space="preserve">https://www.lunduniversity.lu.se</t>
   </si>
   <si>
+    <t xml:space="preserve">71</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://lunduniversity.lu.se/student-life/before-you-arrive/chat-current-students</t>
   </si>
   <si>
@@ -720,6 +762,9 @@
     <t xml:space="preserve">https://www.su.se</t>
   </si>
   <si>
+    <t xml:space="preserve">167</t>
+  </si>
+  <si>
     <t xml:space="preserve">Uppsala University</t>
   </si>
   <si>
@@ -759,6 +804,9 @@
     <t xml:space="preserve">PhD offers usually include tuition and a stipend; most applications close in December.</t>
   </si>
   <si>
+    <t xml:space="preserve">55</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.cmu.edu/ini/admissions/howtoapply.html</t>
   </si>
   <si>
@@ -777,6 +825,9 @@
     <t xml:space="preserve">Mostly December for fall entry – check programme page</t>
   </si>
   <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sangam (Indian students): https://sangam.mit.edu/</t>
   </si>
   <si>
@@ -837,12 +888,294 @@
     <t xml:space="preserve">Set by each department</t>
   </si>
   <si>
+    <t xml:space="preserve">74</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bengali Students Organization (Abol Tabol): https://one.illinois.edu/bengalistudentsorganization/home/</t>
   </si>
   <si>
     <t xml:space="preserve">https://grad.illinois.edu/application-fee</t>
   </si>
   <si>
+    <t xml:space="preserve">Canada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">McGill University</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montreal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mcgill.ca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apply directly to each university (Ontario universities through OUAC): Application fees are usually about CAD 100–160</t>
+  </si>
+  <si>
+    <t xml:space="preserve">About CAD 137 (Fall 2025 figure; check current fee)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Varies by department, e.g. Pathology: 15 Jan (Fall), 1 Aug (Winter) for international applicants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most PhDs are funded through a supervisor or department package; contact potential supervisors early.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mcgill.ca/pathology/programs/apply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of Alberta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edmonton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ualberta.ca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAD 135, non-refundable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Varies by department, e.g. Cell Biology: 1 Jun (Sep start), 1 Oct (Jan start)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">96</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://ualberta.ca/cellbiology/graduate-program/graduate-application-information</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of British Columbia (UBC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vancouver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ubc.ca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fee shown in the application portal; waived for citizens of the UN least developed countries (includes Bangladesh, not India)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set by each programme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://grad.ubc.ca/faq/3240</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of Toronto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toronto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.utoronto.ca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAD 130 (programmes starting Sep 2026–May 2027); CAD 135 (from Sep 2027); no waivers; some programmes add a supplementary fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set by each programme – check the programme page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.sgs.utoronto.ca/admissions/frequently-asked-questions-faqs/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of Waterloo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waterloo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://uwaterloo.ca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAD 150 per programme, non-refundable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set by each programme; apply 2–4 weeks before it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://uwaterloo.ca/future-graduate-students/admissions/how-to-apply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Australia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Australian National University (ANU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canberra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.anu.edu.au</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apply directly to each university: Application fees are usually about AUD 100–155</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUD 150 per application</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semester 1, 2027: 15 Dec 2026 (Crawford School: 31 Oct 2026); Semester 2, 2027: 15 May 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Research degrees (MPhil/PhD) are funded by university and government scholarships; apply to a supervisor first.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://study.anu.edu.au/apply/international-applications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monash University</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.monash.edu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUD 125 for international applicants applying directly (waiver codes at Monash events)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check each course page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.monash.edu/admissions/apply/online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNSW Sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.unsw.edu.au</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of Melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.unimelb.edu.au</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUD 154 per application (waivers only in listed cases, e.g. full sponsorship)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Closing dates on each course's 'How to apply' tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://study.unimelb.edu.au/how-to-apply/fees/application-fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of Sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.sydney.edu.au</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semester 1, 2027: generally 18 Dec 2026 for international postgraduates (some courses differ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leapscholar.com/questions/what-is-the-university-of-sydney-deadline-for-international-postgraduate-applications-for-semester-1-and-2-of-2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">American University of Sharjah (AUS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sharjah</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aus.edu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apply directly to each university: Application fees vary (e.g. Heriot-Watt Dubai AED 525)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026–27 master's: AED 4,371 per credit hour (Arts and Sciences) or AED 5,480 (Engineering, Business, Architecture)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Research universities such as Khalifa University and UAEU offer funded PhD places; check each university.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">258</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.aus.edu/sites/default/files/fall-2026-payment-of-fees-guide-graduate-students-.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heriot-Watt University Dubai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dubai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.hw.ac.uk/dubai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AED 525 (AED 500 + VAT), non-refundable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shown on each programme page; UK degree taught in Dubai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://hw.ac.uk/dubai/study/fees-and-funding/tuition-fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khalifa University</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abu Dhabi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ku.ac.ae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Graduate scholarships for international applicants cover tuition and include a monthly allowance – confirm amounts and deadlines on ku.ac.ae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">147</t>
+  </si>
+  <si>
+    <t xml:space="preserve">United Arab Emirates University (UAEU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Al Ain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.uaeu.ac.ae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Published each year by the College of Graduate Studies (cgs@uaeu.ac.ae)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">217</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.uaeu.ac.ae/en/cgs/</t>
+  </si>
+  <si>
     <t xml:space="preserve">How to apply (undergraduate)</t>
   </si>
   <si>
@@ -913,6 +1246,45 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.commonapp.org/static/ccc61bed5bdc22d15d0054106c6ef52b/Resource_FY_AppFees_ENG_2025.06.25.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apply directly to each university (Ontario universities through OUAC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Application fees are usually about CAD 100–160</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most undergraduate deadlines fall between November and February for September entry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most new students also need a Provincial Attestation Letter; from 1 Jan 2026 master's and PhD students at public universities are exempt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.idp.com/india/blog/visa-rules-for-international-students-canada/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apply directly to each university</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Application fees are usually about AUD 100–155</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two main intakes: February/March (Semester 1) and July (Semester 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tuition is charged per year and varies by course; see each course page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Application fees vary (e.g. Heriot-Watt Dubai AED 525)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most universities admit in autumn and spring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Many Dubai universities are branch campuses of UK, Australian or Indian universities; check that the degree is recognised where you want to work</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://gulfnews.com/uae/indian-students-top-dubais-global-intake-at-43-pakistanis-at-6-1.500190286</t>
   </si>
 </sst>
 </file>
@@ -1171,9 +1543,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Universities" displayName="Universities" ref="A1:O36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O36"/>
-  <tableColumns count="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Universities" displayName="Universities" ref="A1:P50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:P50"/>
+  <tableColumns count="16">
     <tableColumn id="1" name="Country"/>
     <tableColumn id="2" name="University"/>
     <tableColumn id="3" name="City"/>
@@ -1184,11 +1556,12 @@
     <tableColumn id="8" name="Example tuition (international)"/>
     <tableColumn id="9" name="Scholarships for India / Bangladesh"/>
     <tableColumn id="10" name="PhD – how it works"/>
-    <tableColumn id="11" name="Chat with current students"/>
-    <tableColumn id="12" name="Indian / Bengali / Bangladeshi societies"/>
-    <tableColumn id="13" name="Country pages"/>
-    <tableColumn id="14" name="Sources"/>
-    <tableColumn id="15" name="Checked"/>
+    <tableColumn id="11" name="QS World University Rankings 2027"/>
+    <tableColumn id="12" name="Chat with current students"/>
+    <tableColumn id="13" name="Indian / Bengali / Bangladeshi societies"/>
+    <tableColumn id="14" name="Country pages"/>
+    <tableColumn id="15" name="Sources"/>
+    <tableColumn id="16" name="Checked"/>
   </tableColumns>
 </table>
 </file>
@@ -1464,7 +1837,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:P50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -1474,14 +1847,16 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="9" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
         <v>12</v>
       </c>
@@ -1527,1376 +1902,2042 @@
       <c r="O1" s="6" t="s">
         <v>26</v>
       </c>
+      <c r="P1" s="6" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F2" s="7"/>
       <c r="G2" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
       <c r="J2" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="L2" s="7"/>
+        <v>35</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>36</v>
+      </c>
       <c r="M2" s="7"/>
-      <c r="N2" s="7" t="s">
-        <v>35</v>
-      </c>
+      <c r="N2" s="7"/>
       <c r="O2" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="P2" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="M3" s="7"/>
-      <c r="N3" s="7" t="s">
-        <v>44</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="N3" s="7"/>
       <c r="O3" s="7" t="s">
-        <v>36</v>
+        <v>47</v>
+      </c>
+      <c r="P3" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
       <c r="I4" s="7"/>
       <c r="J4" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>49</v>
+        <v>34</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <f aca="false">2</f>
+        <v>2</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7" t="s">
-        <v>51</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="N4" s="7"/>
       <c r="O4" s="7" t="s">
-        <v>36</v>
+        <v>54</v>
+      </c>
+      <c r="P4" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="I5" s="7"/>
       <c r="J5" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="M5" s="7"/>
-      <c r="N5" s="7" t="s">
-        <v>59</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N5" s="7"/>
       <c r="O5" s="7" t="s">
-        <v>36</v>
+        <v>63</v>
+      </c>
+      <c r="P5" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G6" s="7"/>
       <c r="H6" s="7"/>
       <c r="I6" s="7"/>
       <c r="J6" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>36</v>
+        <v>71</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="L7" s="7"/>
+        <v>35</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>76</v>
+      </c>
       <c r="M7" s="7"/>
-      <c r="N7" s="7" t="s">
-        <v>72</v>
-      </c>
+      <c r="N7" s="7"/>
       <c r="O7" s="7" t="s">
-        <v>36</v>
+        <v>77</v>
+      </c>
+      <c r="P7" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H8" s="7"/>
       <c r="I8" s="7" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="L8" s="7"/>
+        <v>35</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>83</v>
+      </c>
       <c r="M8" s="7"/>
-      <c r="N8" s="7" t="s">
-        <v>79</v>
-      </c>
+      <c r="N8" s="7"/>
       <c r="O8" s="7" t="s">
-        <v>36</v>
+        <v>84</v>
+      </c>
+      <c r="P8" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
       <c r="I9" s="7"/>
       <c r="J9" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>83</v>
+        <v>34</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <f aca="false">8</f>
+        <v>8</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7" t="s">
-        <v>85</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="N9" s="7"/>
       <c r="O9" s="7" t="s">
-        <v>36</v>
+        <v>90</v>
+      </c>
+      <c r="P9" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="H10" s="7"/>
       <c r="I10" s="7"/>
       <c r="J10" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="K10" s="7" t="s">
-        <v>91</v>
+        <v>34</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <f aca="false">68</f>
+        <v>68</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7" t="s">
-        <v>93</v>
-      </c>
+        <v>96</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="N10" s="7"/>
       <c r="O10" s="7" t="s">
-        <v>36</v>
+        <v>98</v>
+      </c>
+      <c r="P10" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
       <c r="I11" s="7"/>
       <c r="J11" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="M11" s="7"/>
-      <c r="N11" s="7" t="s">
-        <v>100</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="N11" s="7"/>
       <c r="O11" s="7" t="s">
-        <v>36</v>
+        <v>106</v>
+      </c>
+      <c r="P11" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="H12" s="7"/>
       <c r="I12" s="7" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7" t="s">
-        <v>110</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="M12" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="N12" s="7"/>
       <c r="O12" s="7" t="s">
-        <v>36</v>
+        <v>117</v>
+      </c>
+      <c r="P12" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
       <c r="I13" s="7"/>
       <c r="J13" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="L13" s="7"/>
+        <v>122</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>123</v>
+      </c>
       <c r="M13" s="7"/>
       <c r="N13" s="7"/>
-      <c r="O13" s="7" t="s">
-        <v>36</v>
+      <c r="O13" s="7"/>
+      <c r="P13" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="H14" s="7"/>
       <c r="I14" s="7"/>
       <c r="J14" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="L14" s="7"/>
+        <v>129</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>130</v>
+      </c>
       <c r="M14" s="7"/>
-      <c r="N14" s="7" t="s">
-        <v>122</v>
-      </c>
+      <c r="N14" s="7"/>
       <c r="O14" s="7" t="s">
-        <v>36</v>
+        <v>131</v>
+      </c>
+      <c r="P14" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="H15" s="7"/>
       <c r="I15" s="7"/>
       <c r="J15" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="K15" s="7" t="s">
-        <v>127</v>
+        <v>34</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <f aca="false">77</f>
+        <v>77</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="M15" s="7"/>
-      <c r="N15" s="7" t="s">
-        <v>129</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="N15" s="7"/>
       <c r="O15" s="7" t="s">
-        <v>36</v>
+        <v>138</v>
+      </c>
+      <c r="P15" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="I16" s="7"/>
       <c r="J16" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="K16" s="7" t="s">
-        <v>136</v>
+        <v>34</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <f aca="false">40</f>
+        <v>40</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="N16" s="7" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="O16" s="7" t="s">
-        <v>36</v>
+        <v>148</v>
+      </c>
+      <c r="P16" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="H17" s="7"/>
       <c r="I17" s="7"/>
       <c r="J17" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="K17" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="L17" s="7"/>
+        <v>34</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <f aca="false">97</f>
+        <v>97</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>154</v>
+      </c>
       <c r="M17" s="7"/>
-      <c r="N17" s="7" t="s">
-        <v>146</v>
-      </c>
+      <c r="N17" s="7"/>
       <c r="O17" s="7" t="s">
-        <v>36</v>
+        <v>155</v>
+      </c>
+      <c r="P17" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="H18" s="7"/>
       <c r="I18" s="7"/>
       <c r="J18" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="L18" s="7"/>
+        <v>161</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>162</v>
+      </c>
       <c r="M18" s="7"/>
-      <c r="N18" s="7" t="s">
-        <v>153</v>
-      </c>
+      <c r="N18" s="7"/>
       <c r="O18" s="7" t="s">
-        <v>36</v>
+        <v>163</v>
+      </c>
+      <c r="P18" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
       <c r="I19" s="7" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="K19" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="L19" s="7"/>
+        <v>34</v>
+      </c>
+      <c r="K19" s="7" t="n">
+        <f aca="false">82</f>
+        <v>82</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>169</v>
+      </c>
       <c r="M19" s="7"/>
-      <c r="N19" s="7" t="s">
-        <v>160</v>
-      </c>
+      <c r="N19" s="7"/>
       <c r="O19" s="7" t="s">
-        <v>36</v>
+        <v>170</v>
+      </c>
+      <c r="P19" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="H20" s="7"/>
       <c r="I20" s="7"/>
       <c r="J20" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>166</v>
+        <v>35</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="M20" s="7"/>
-      <c r="N20" s="7" t="s">
-        <v>168</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="N20" s="7"/>
       <c r="O20" s="7" t="s">
-        <v>36</v>
+        <v>178</v>
+      </c>
+      <c r="P20" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="H21" s="7"/>
       <c r="I21" s="7"/>
       <c r="J21" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="K21" s="7" t="s">
-        <v>173</v>
+        <v>34</v>
+      </c>
+      <c r="K21" s="7" t="n">
+        <f aca="false">68</f>
+        <v>68</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="M21" s="7"/>
-      <c r="N21" s="7" t="s">
-        <v>175</v>
-      </c>
+        <v>183</v>
+      </c>
+      <c r="M21" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="N21" s="7"/>
       <c r="O21" s="7" t="s">
-        <v>36</v>
+        <v>185</v>
+      </c>
+      <c r="P21" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="F22" s="7"/>
       <c r="G22" s="7" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="I22" s="7"/>
       <c r="J22" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="K22" s="7"/>
+        <v>193</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>194</v>
+      </c>
       <c r="L22" s="7"/>
       <c r="M22" s="7"/>
-      <c r="N22" s="7" t="s">
-        <v>184</v>
-      </c>
+      <c r="N22" s="7"/>
       <c r="O22" s="7" t="s">
-        <v>36</v>
+        <v>195</v>
+      </c>
+      <c r="P22" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="F23" s="7"/>
       <c r="G23" s="7" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="I23" s="7"/>
       <c r="J23" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="K23" s="7"/>
-      <c r="L23" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="M23" s="7"/>
-      <c r="N23" s="7" t="s">
-        <v>191</v>
-      </c>
+        <v>193</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="L23" s="7"/>
+      <c r="M23" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="N23" s="7"/>
       <c r="O23" s="7" t="s">
-        <v>36</v>
+        <v>203</v>
+      </c>
+      <c r="P23" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="F24" s="7"/>
       <c r="G24" s="7" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="I24" s="7"/>
       <c r="J24" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="K24" s="7"/>
-      <c r="L24" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="M24" s="7"/>
-      <c r="N24" s="7" t="s">
-        <v>198</v>
-      </c>
+        <v>193</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="L24" s="7"/>
+      <c r="M24" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="N24" s="7"/>
       <c r="O24" s="7" t="s">
-        <v>36</v>
+        <v>210</v>
+      </c>
+      <c r="P24" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="I25" s="7"/>
       <c r="J25" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="K25" s="7"/>
+        <v>193</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>35</v>
+      </c>
       <c r="L25" s="7"/>
       <c r="M25" s="7"/>
-      <c r="N25" s="7" t="s">
-        <v>205</v>
-      </c>
+      <c r="N25" s="7"/>
       <c r="O25" s="7" t="s">
-        <v>36</v>
+        <v>217</v>
+      </c>
+      <c r="P25" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="F26" s="7"/>
       <c r="G26" s="7" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="I26" s="7"/>
       <c r="J26" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="M26" s="7"/>
-      <c r="N26" s="7" t="s">
-        <v>210</v>
-      </c>
+        <v>193</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="L26" s="7"/>
+      <c r="M26" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="N26" s="7"/>
       <c r="O26" s="7" t="s">
-        <v>36</v>
+        <v>223</v>
+      </c>
+      <c r="P26" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="H27" s="7"/>
       <c r="I27" s="7"/>
       <c r="J27" s="7" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="L27" s="7"/>
+        <v>35</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>232</v>
+      </c>
       <c r="M27" s="7"/>
       <c r="N27" s="7"/>
-      <c r="O27" s="7" t="s">
-        <v>36</v>
+      <c r="O27" s="7"/>
+      <c r="P27" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="H28" s="7"/>
       <c r="I28" s="7"/>
       <c r="J28" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="K28" s="7"/>
+        <v>231</v>
+      </c>
+      <c r="K28" s="7" t="n">
+        <f aca="false">82</f>
+        <v>82</v>
+      </c>
       <c r="L28" s="7"/>
       <c r="M28" s="7"/>
-      <c r="N28" s="7" t="s">
-        <v>225</v>
-      </c>
+      <c r="N28" s="7"/>
       <c r="O28" s="7" t="s">
-        <v>36</v>
+        <v>238</v>
+      </c>
+      <c r="P28" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="D29" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="E29" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="E29" s="7" t="s">
-        <v>215</v>
-      </c>
       <c r="F29" s="7" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="H29" s="7"/>
       <c r="I29" s="7"/>
       <c r="J29" s="7" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="L29" s="7"/>
+        <v>242</v>
+      </c>
+      <c r="L29" s="7" t="s">
+        <v>243</v>
+      </c>
       <c r="M29" s="7"/>
-      <c r="N29" s="7" t="s">
-        <v>225</v>
-      </c>
+      <c r="N29" s="7"/>
       <c r="O29" s="7" t="s">
-        <v>36</v>
+        <v>238</v>
+      </c>
+      <c r="P29" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="B30" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="G30" s="7" t="s">
         <v>230</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="D30" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="E30" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>217</v>
       </c>
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="K30" s="7"/>
+        <v>231</v>
+      </c>
+      <c r="K30" s="7" t="s">
+        <v>246</v>
+      </c>
       <c r="L30" s="7"/>
       <c r="M30" s="7"/>
       <c r="N30" s="7"/>
-      <c r="O30" s="7" t="s">
-        <v>36</v>
+      <c r="O30" s="7"/>
+      <c r="P30" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>232</v>
+        <v>247</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="K31" s="7" t="s">
-        <v>235</v>
-      </c>
-      <c r="L31" s="7"/>
+        <v>231</v>
+      </c>
+      <c r="K31" s="7" t="n">
+        <f aca="false">87</f>
+        <v>87</v>
+      </c>
+      <c r="L31" s="7" t="s">
+        <v>250</v>
+      </c>
       <c r="M31" s="7"/>
       <c r="N31" s="7"/>
-      <c r="O31" s="7" t="s">
-        <v>36</v>
+      <c r="O31" s="7"/>
+      <c r="P31" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>237</v>
+        <v>252</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>238</v>
+        <v>253</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="H32" s="7" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
       <c r="I32" s="7"/>
       <c r="J32" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="K32" s="7"/>
+        <v>259</v>
+      </c>
+      <c r="K32" s="7" t="s">
+        <v>260</v>
+      </c>
       <c r="L32" s="7"/>
       <c r="M32" s="7"/>
-      <c r="N32" s="7" t="s">
-        <v>245</v>
-      </c>
+      <c r="N32" s="7"/>
       <c r="O32" s="7" t="s">
-        <v>36</v>
+        <v>261</v>
+      </c>
+      <c r="P32" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>246</v>
+        <v>262</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>248</v>
+        <v>264</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>249</v>
+        <v>265</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>250</v>
+        <v>266</v>
       </c>
       <c r="H33" s="7"/>
       <c r="I33" s="7"/>
       <c r="J33" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="K33" s="7"/>
-      <c r="L33" s="7" t="s">
-        <v>251</v>
-      </c>
-      <c r="M33" s="7"/>
-      <c r="N33" s="7" t="s">
-        <v>252</v>
-      </c>
+        <v>259</v>
+      </c>
+      <c r="K33" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="L33" s="7"/>
+      <c r="M33" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="N33" s="7"/>
       <c r="O33" s="7" t="s">
-        <v>36</v>
+        <v>269</v>
+      </c>
+      <c r="P33" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>253</v>
+        <v>270</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>254</v>
+        <v>271</v>
       </c>
       <c r="D34" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="E34" s="7" t="s">
         <v>255</v>
       </c>
-      <c r="E34" s="7" t="s">
-        <v>240</v>
-      </c>
       <c r="F34" s="7" t="s">
-        <v>256</v>
+        <v>273</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>257</v>
+        <v>274</v>
       </c>
       <c r="H34" s="7"/>
       <c r="I34" s="7"/>
       <c r="J34" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="K34" s="7"/>
-      <c r="L34" s="7" t="s">
-        <v>258</v>
-      </c>
-      <c r="M34" s="7"/>
-      <c r="N34" s="7" t="s">
         <v>259</v>
       </c>
+      <c r="K34" s="7" t="n">
+        <f aca="false">100</f>
+        <v>100</v>
+      </c>
+      <c r="L34" s="7"/>
+      <c r="M34" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="N34" s="7"/>
       <c r="O34" s="7" t="s">
-        <v>36</v>
+        <v>276</v>
+      </c>
+      <c r="P34" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>260</v>
+        <v>277</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>261</v>
+        <v>278</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>262</v>
+        <v>279</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>263</v>
+        <v>280</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>264</v>
+        <v>281</v>
       </c>
       <c r="H35" s="7"/>
       <c r="I35" s="7"/>
       <c r="J35" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="K35" s="7"/>
+        <v>259</v>
+      </c>
+      <c r="K35" s="7" t="n">
+        <f aca="false">2</f>
+        <v>2</v>
+      </c>
       <c r="L35" s="7"/>
       <c r="M35" s="7"/>
-      <c r="N35" s="7" t="s">
-        <v>265</v>
-      </c>
+      <c r="N35" s="7"/>
       <c r="O35" s="7" t="s">
-        <v>36</v>
+        <v>282</v>
+      </c>
+      <c r="P35" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>266</v>
+        <v>283</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>267</v>
+        <v>284</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>268</v>
+        <v>285</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>269</v>
+        <v>286</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>270</v>
+        <v>287</v>
       </c>
       <c r="H36" s="7"/>
       <c r="I36" s="7"/>
       <c r="J36" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="K36" s="7"/>
-      <c r="L36" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="M36" s="7"/>
-      <c r="N36" s="7" t="s">
-        <v>272</v>
-      </c>
+        <v>259</v>
+      </c>
+      <c r="K36" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="L36" s="7"/>
+      <c r="M36" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="N36" s="7"/>
       <c r="O36" s="7" t="s">
-        <v>36</v>
+        <v>290</v>
+      </c>
+      <c r="P36" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="H37" s="7"/>
+      <c r="I37" s="7"/>
+      <c r="J37" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="K37" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="L37" s="7"/>
+      <c r="M37" s="7"/>
+      <c r="N37" s="7"/>
+      <c r="O37" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="P37" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="H38" s="7"/>
+      <c r="I38" s="7"/>
+      <c r="J38" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="K38" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="L38" s="7"/>
+      <c r="M38" s="7"/>
+      <c r="N38" s="7"/>
+      <c r="O38" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="P38" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="H39" s="7"/>
+      <c r="I39" s="7"/>
+      <c r="J39" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="K39" s="7" t="n">
+        <f aca="false">45</f>
+        <v>45</v>
+      </c>
+      <c r="L39" s="7"/>
+      <c r="M39" s="7"/>
+      <c r="N39" s="7"/>
+      <c r="O39" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="P39" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>318</v>
+      </c>
+      <c r="H40" s="7"/>
+      <c r="I40" s="7"/>
+      <c r="J40" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="K40" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="L40" s="7"/>
+      <c r="M40" s="7"/>
+      <c r="N40" s="7"/>
+      <c r="O40" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="P40" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="H41" s="7"/>
+      <c r="I41" s="7"/>
+      <c r="J41" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="K41" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="L41" s="7"/>
+      <c r="M41" s="7"/>
+      <c r="N41" s="7"/>
+      <c r="O41" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="P41" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="G42" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="H42" s="7"/>
+      <c r="I42" s="7"/>
+      <c r="J42" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="K42" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="L42" s="7"/>
+      <c r="M42" s="7"/>
+      <c r="N42" s="7"/>
+      <c r="O42" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="P42" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>340</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>341</v>
+      </c>
+      <c r="H43" s="7"/>
+      <c r="I43" s="7"/>
+      <c r="J43" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="K43" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="L43" s="7"/>
+      <c r="M43" s="7"/>
+      <c r="N43" s="7"/>
+      <c r="O43" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="P43" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="F44" s="7"/>
+      <c r="G44" s="7" t="s">
+        <v>341</v>
+      </c>
+      <c r="H44" s="7"/>
+      <c r="I44" s="7"/>
+      <c r="J44" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="K44" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="L44" s="7"/>
+      <c r="M44" s="7"/>
+      <c r="N44" s="7"/>
+      <c r="O44" s="7"/>
+      <c r="P44" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="G45" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="H45" s="7"/>
+      <c r="I45" s="7"/>
+      <c r="J45" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="K45" s="7" t="n">
+        <f aca="false">22</f>
+        <v>22</v>
+      </c>
+      <c r="L45" s="7"/>
+      <c r="M45" s="7"/>
+      <c r="N45" s="7"/>
+      <c r="O45" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="P45" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>354</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="F46" s="7"/>
+      <c r="G46" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="H46" s="7"/>
+      <c r="I46" s="7"/>
+      <c r="J46" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="K46" s="7" t="s">
+        <v>356</v>
+      </c>
+      <c r="L46" s="7"/>
+      <c r="M46" s="7"/>
+      <c r="N46" s="7"/>
+      <c r="O46" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="P46" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="7" t="s">
+        <v>363</v>
+      </c>
+      <c r="I47" s="7"/>
+      <c r="J47" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="K47" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="L47" s="7"/>
+      <c r="M47" s="7"/>
+      <c r="N47" s="7"/>
+      <c r="O47" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="P47" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="E48" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>370</v>
+      </c>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="I48" s="7"/>
+      <c r="J48" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="K48" s="7"/>
+      <c r="L48" s="7"/>
+      <c r="M48" s="7"/>
+      <c r="N48" s="7"/>
+      <c r="O48" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="P48" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>374</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="J49" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="K49" s="7" t="s">
+        <v>377</v>
+      </c>
+      <c r="L49" s="7"/>
+      <c r="M49" s="7"/>
+      <c r="N49" s="7"/>
+      <c r="O49" s="7"/>
+      <c r="P49" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>378</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="D50" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="E50" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="H50" s="7"/>
+      <c r="I50" s="7"/>
+      <c r="J50" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="K50" s="7" t="s">
+        <v>382</v>
+      </c>
+      <c r="L50" s="7"/>
+      <c r="M50" s="7"/>
+      <c r="N50" s="7"/>
+      <c r="O50" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="P50" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -2918,7 +3959,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -2934,129 +3975,210 @@
         <v>12</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>273</v>
+        <v>384</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>274</v>
+        <v>385</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>275</v>
+        <v>386</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>276</v>
+        <v>387</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>277</v>
+        <v>388</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>278</v>
+        <v>389</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>279</v>
+        <v>390</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>280</v>
+        <v>391</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>281</v>
+        <v>392</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>282</v>
+        <v>393</v>
       </c>
       <c r="E2" s="7"/>
       <c r="F2" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G2" s="7" t="n">
-        <f aca="false">COUNTIF(Universities!$A$2:$A$36,A2)</f>
+        <f aca="false">COUNTIF(Universities!$A$2:$A$50,A2)</f>
         <v>20</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>283</v>
+        <v>394</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>284</v>
+        <v>395</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>285</v>
+        <v>396</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>286</v>
+        <v>397</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>287</v>
+        <v>398</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="G3" s="7" t="n">
-        <f aca="false">COUNTIF(Universities!$A$2:$A$36,A3)</f>
+        <f aca="false">COUNTIF(Universities!$A$2:$A$50,A3)</f>
         <v>5</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>288</v>
+        <v>399</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>289</v>
+        <v>400</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>290</v>
+        <v>401</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>291</v>
+        <v>402</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>292</v>
+        <v>403</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="G4" s="7" t="n">
-        <f aca="false">COUNTIF(Universities!$A$2:$A$36,A4)</f>
+        <f aca="false">COUNTIF(Universities!$A$2:$A$50,A4)</f>
         <v>5</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>293</v>
+        <v>404</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>294</v>
+        <v>405</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>295</v>
+        <v>406</v>
       </c>
       <c r="E5" s="7"/>
       <c r="F5" s="7" t="s">
-        <v>244</v>
+        <v>259</v>
       </c>
       <c r="G5" s="7" t="n">
-        <f aca="false">COUNTIF(Universities!$A$2:$A$36,A5)</f>
+        <f aca="false">COUNTIF(Universities!$A$2:$A$50,A5)</f>
         <v>5</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>296</v>
+        <v>407</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <f aca="false">COUNTIF(Universities!$A$2:$A$50,A6)</f>
+        <v>5</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>414</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>415</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <f aca="false">COUNTIF(Universities!$A$2:$A$50,A7)</f>
+        <v>5</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>417</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>418</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>419</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <f aca="false">COUNTIF(Universities!$A$2:$A$50,A8)</f>
+        <v>4</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>420</v>
       </c>
     </row>
   </sheetData>

</xml_diff>